<commit_message>
Update Cataleg: data files and app changes
Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Cataleg/jerarquia.xlsx
+++ b/Cataleg/jerarquia.xlsx
@@ -22497,8 +22497,8 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x0101002608A4117A73EF40A68248878EC111FD" ma:contentTypeVersion="13" ma:contentTypeDescription="Crea un document nou" ma:contentTypeScope="" ma:versionID="b79346ae0e0a813eceff9ed4fc9eeadd">
-  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="c40011fc-6905-4b98-896a-b89e6ed00ba6" xmlns:ns3="44e8012d-71fe-413e-9307-5fe54acf1bd3" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="ae86b347dfc234c70f83e507845b4195" ns2:_="" ns3:_="">
+<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x0101002608A4117A73EF40A68248878EC111FD" ma:contentTypeVersion="14" ma:contentTypeDescription="Crea un document nou" ma:contentTypeScope="" ma:versionID="0cfb8dfb04eab00c53cc8369037f759e">
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="c40011fc-6905-4b98-896a-b89e6ed00ba6" xmlns:ns3="44e8012d-71fe-413e-9307-5fe54acf1bd3" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="a6fd102206446d69fbc6a91a53858934" ns2:_="" ns3:_="">
     <xsd:import namespace="c40011fc-6905-4b98-896a-b89e6ed00ba6"/>
     <xsd:import namespace="44e8012d-71fe-413e-9307-5fe54acf1bd3"/>
     <xsd:element name="properties">
@@ -22519,6 +22519,7 @@
                 <xsd:element ref="ns2:MediaLengthInSeconds" minOccurs="0"/>
                 <xsd:element ref="ns2:MediaServiceObjectDetectorVersions" minOccurs="0"/>
                 <xsd:element ref="ns2:MediaServiceSearchProperties" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceDateTaken" minOccurs="0"/>
               </xsd:all>
             </xsd:complexType>
           </xsd:element>
@@ -22576,6 +22577,11 @@
     <xsd:element name="MediaServiceSearchProperties" ma:index="20" nillable="true" ma:displayName="MediaServiceSearchProperties" ma:hidden="true" ma:internalName="MediaServiceSearchProperties" ma:readOnly="true">
       <xsd:simpleType>
         <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceDateTaken" ma:index="21" nillable="true" ma:displayName="MediaServiceDateTaken" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceDateTaken" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
       </xsd:simpleType>
     </xsd:element>
   </xsd:schema>
@@ -22740,7 +22746,7 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{4A76C969-209E-4186-B911-68DE37B73FF9}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{398D1BB2-923D-475C-990E-A865B017E7C6}"/>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>

</xml_diff>